<commit_message>
Added IMAP workflow to verify successful connection
</commit_message>
<xml_diff>
--- a/Data/Testdata/Unittests.xlsx
+++ b/Data/Testdata/Unittests.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\Testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C521B79-CB7E-4D36-923C-1A2E66DF2C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33EA5381-3BAA-47C0-9EAA-88DAD961B488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11835" xr2:uid="{0F59387B-8167-4962-A8A1-49C75F9DA195}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{0F59387B-8167-4962-A8A1-49C75F9DA195}"/>
   </bookViews>
   <sheets>
     <sheet name="OpenBrowser" sheetId="1" r:id="rId1"/>
+    <sheet name="VerifyImapConn" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
   <si>
     <t>in_Environment</t>
   </si>
@@ -46,6 +47,18 @@
   </si>
   <si>
     <t>true</t>
+  </si>
+  <si>
+    <t>dev</t>
+  </si>
+  <si>
+    <t>in_ConfigFile</t>
+  </si>
+  <si>
+    <t>Data\Config_Dev.xlsx</t>
+  </si>
+  <si>
+    <t>in_MinMailmsgsCountExpected</t>
   </si>
 </sst>
 </file>
@@ -444,4 +457,47 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADAA743D-90C4-4034-A07B-93BE2630C4A8}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Implemented TestCase for config items. WIP #11
</commit_message>
<xml_diff>
--- a/Data/Testdata/Unittests.xlsx
+++ b/Data/Testdata/Unittests.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\Testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33EA5381-3BAA-47C0-9EAA-88DAD961B488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD09FED0-44E4-439E-8157-A0BED2EB5D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{0F59387B-8167-4962-A8A1-49C75F9DA195}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11835" activeTab="2" xr2:uid="{0F59387B-8167-4962-A8A1-49C75F9DA195}"/>
   </bookViews>
   <sheets>
     <sheet name="OpenBrowser" sheetId="1" r:id="rId1"/>
     <sheet name="VerifyImapConn" sheetId="2" r:id="rId2"/>
+    <sheet name="Config" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="28">
   <si>
     <t>in_Environment</t>
   </si>
@@ -59,6 +60,66 @@
   </si>
   <si>
     <t>in_MinMailmsgsCountExpected</t>
+  </si>
+  <si>
+    <t>OrchestratorFolderPath</t>
+  </si>
+  <si>
+    <t>logF_BusinessProcessName</t>
+  </si>
+  <si>
+    <t>QueueConsumptionStrategy</t>
+  </si>
+  <si>
+    <t>Imap_Server</t>
+  </si>
+  <si>
+    <t>Imap_Port</t>
+  </si>
+  <si>
+    <t>Imap_Credentialname</t>
+  </si>
+  <si>
+    <t>Mailbox_FolderIncoming</t>
+  </si>
+  <si>
+    <t>Mailbox_Batchsize</t>
+  </si>
+  <si>
+    <t>Mailbox_FolderProcessing</t>
+  </si>
+  <si>
+    <t>Mailbox_FolderHandover2Human</t>
+  </si>
+  <si>
+    <t>Mailbox_FolderSuccessful</t>
+  </si>
+  <si>
+    <t>File_BasePathTemp</t>
+  </si>
+  <si>
+    <t>FTP_ServerHostname</t>
+  </si>
+  <si>
+    <t>FTP_ServerPort</t>
+  </si>
+  <si>
+    <t>FTP_CredentialName</t>
+  </si>
+  <si>
+    <t>FTP_RemotePathPristine</t>
+  </si>
+  <si>
+    <t>FTP_RemotePathTainted</t>
+  </si>
+  <si>
+    <t>in_ConfigItem</t>
+  </si>
+  <si>
+    <t>foo</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
 </sst>
 </file>
@@ -500,4 +561,284 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FD2DB8F-8CD4-4CCE-9F1A-7FED9B15A02E}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added end-to-end TestCase executing Main.xaml with varying in_ConfigPath
</commit_message>
<xml_diff>
--- a/Data/Testdata/Unittests.xlsx
+++ b/Data/Testdata/Unittests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\PurposefulPromethium\Data\Testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD09FED0-44E4-439E-8157-A0BED2EB5D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{512FF058-1FD6-4E57-92F0-A52486132947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11835" activeTab="2" xr2:uid="{0F59387B-8167-4962-A8A1-49C75F9DA195}"/>
+    <workbookView xWindow="1575" yWindow="4065" windowWidth="21600" windowHeight="11835" activeTab="2" xr2:uid="{0F59387B-8167-4962-A8A1-49C75F9DA195}"/>
   </bookViews>
   <sheets>
     <sheet name="OpenBrowser" sheetId="1" r:id="rId1"/>

</xml_diff>